<commit_message>
feat: add clubs, emergency status, kindergarten history, and UI improvements
- Clubs system (4 clubs with attendance, checkin, dashboard, history calendar)
- Emergency status for 634 residents (4 status types, pagination, export)
- Kindergarten history with daily calendar snapshots
- Shelter history with calendar view per shelter
- Issues & distress history with calendar + search
- Bottom nav with all tabs, active tab highlighting
- Export buttons (email/WhatsApp → PDF/Excel/both)
- 2-column shelter grid, fixed images, centered titles
- SOS button blinks on active alerts
- Renamed emergency tab to "עדכון תושבים"

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/src/assets/distress/טבלת גנים.xlsx
+++ b/src/assets/distress/טבלת גנים.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/dba97155a5237de2/שולחן העבודה/חרבות ברזל - צרעה/צרעה/אפליקציה/גנים/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guy\OneDrive\claude\status\src\assets\distress\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="182" documentId="8_{9F6EFDF8-D254-4107-ACE5-E6A86D1C60A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0F07FC36-F75C-4582-BD1F-70D55350A676}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0D3BCBF-6EAA-4120-ABFE-2CC8D21BB8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13992" activeTab="5" xr2:uid="{DA12C325-302C-469F-A99F-A5D66028FFAC}"/>
+    <workbookView xWindow="-30855" yWindow="1350" windowWidth="21600" windowHeight="10560" activeTab="2" xr2:uid="{DA12C325-302C-469F-A99F-A5D66028FFAC}"/>
   </bookViews>
   <sheets>
     <sheet name="בית תינוקות" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="153">
   <si>
     <t>משפחה</t>
   </si>
@@ -407,12 +407,108 @@
   </si>
   <si>
     <t>איתן שעני</t>
+  </si>
+  <si>
+    <t>שיר גן גזובסקי</t>
+  </si>
+  <si>
+    <t>נאוה צור</t>
+  </si>
+  <si>
+    <t>ניקול אקשטיין</t>
+  </si>
+  <si>
+    <t>בת חן אסרף</t>
+  </si>
+  <si>
+    <t>מרגלית צברי</t>
+  </si>
+  <si>
+    <t>בת שבע אשרף</t>
+  </si>
+  <si>
+    <t>עפר קריב</t>
+  </si>
+  <si>
+    <t>סגל חינוכי</t>
+  </si>
+  <si>
+    <t>יולנדה ל בורמן</t>
+  </si>
+  <si>
+    <t>רות אקרלינג</t>
+  </si>
+  <si>
+    <t>ורד רפפורט</t>
+  </si>
+  <si>
+    <t>דורית כהן</t>
+  </si>
+  <si>
+    <t>סימה רגב</t>
+  </si>
+  <si>
+    <t>הודא נבאברה</t>
+  </si>
+  <si>
+    <t>ליעד שטיין</t>
+  </si>
+  <si>
+    <t>מאיה פלאוט</t>
+  </si>
+  <si>
+    <t>קרן אוזינסקי</t>
+  </si>
+  <si>
+    <t>תמר ששון נדלר</t>
+  </si>
+  <si>
+    <t>שקד שרה אלמליח</t>
+  </si>
+  <si>
+    <t>טל שירה ששון</t>
+  </si>
+  <si>
+    <t>אסתר משילקר</t>
+  </si>
+  <si>
+    <t>זיו יהב</t>
+  </si>
+  <si>
+    <t>נטע שגיא</t>
+  </si>
+  <si>
+    <t>אלה לפידות</t>
+  </si>
+  <si>
+    <t>ליאורה לוי</t>
+  </si>
+  <si>
+    <t>מישל ווקנין</t>
+  </si>
+  <si>
+    <t>זנבו גטו</t>
+  </si>
+  <si>
+    <t>סארה נבאברה</t>
+  </si>
+  <si>
+    <t>אלישבע ברסטצקי</t>
+  </si>
+  <si>
+    <t>שיר בודנהימר</t>
+  </si>
+  <si>
+    <t>איילה ימין</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="#0.0"/>
+  </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -518,10 +614,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -856,18 +952,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97458083-0E93-46DC-B44A-46473F6F6D7D}">
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:C10"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.6171875" customWidth="1"/>
+    <col min="3" max="3" width="9.875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
     </row>
-    <row r="2" spans="1:3" s="5" customFormat="1" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:3" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>16</v>
       </c>
@@ -875,7 +971,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="9">
         <v>1</v>
       </c>
@@ -886,7 +982,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
         <v>2</v>
       </c>
@@ -897,7 +993,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" ht="28.5" x14ac:dyDescent="0.2">
       <c r="A5" s="9">
         <v>3</v>
       </c>
@@ -908,7 +1004,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="8">
         <v>4</v>
       </c>
@@ -919,7 +1015,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="9">
         <v>5</v>
       </c>
@@ -930,7 +1026,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
         <v>6</v>
       </c>
@@ -941,8 +1037,8 @@
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A9" s="11">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="8">
         <v>7</v>
       </c>
       <c r="B9" s="6" t="s">
@@ -952,8 +1048,8 @@
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A10" s="11">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="8">
         <v>8</v>
       </c>
       <c r="B10" s="6" t="s">
@@ -962,9 +1058,6 @@
       <c r="C10" s="7" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A11" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -976,17 +1069,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F841B40-6139-4762-A084-04C72FBE76E4}">
-  <dimension ref="A1:C15"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="15.80859375" customWidth="1"/>
+    <col min="3" max="3" width="15.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
     </row>
-    <row r="2" spans="1:3" s="5" customFormat="1" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:3" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>16</v>
       </c>
@@ -994,7 +1087,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="8">
         <v>1</v>
       </c>
@@ -1005,7 +1098,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
         <v>2</v>
       </c>
@@ -1016,7 +1109,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="8">
         <v>3</v>
       </c>
@@ -1027,7 +1120,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="8">
         <v>4</v>
       </c>
@@ -1038,7 +1131,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="8">
         <v>5</v>
       </c>
@@ -1049,7 +1142,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
         <v>6</v>
       </c>
@@ -1060,7 +1153,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
         <v>7</v>
       </c>
@@ -1071,7 +1164,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
         <v>8</v>
       </c>
@@ -1082,8 +1175,8 @@
         <v>25</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A11" s="11">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="8">
         <v>9</v>
       </c>
       <c r="B11" s="6" t="s">
@@ -1093,8 +1186,8 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A12" s="11">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="8">
         <v>10</v>
       </c>
       <c r="B12" s="6" t="s">
@@ -1104,8 +1197,8 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A13" s="11">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="8">
         <v>11</v>
       </c>
       <c r="B13" s="6" t="s">
@@ -1114,12 +1207,6 @@
       <c r="C13" s="7" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A14" s="12"/>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A15" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1131,17 +1218,17 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7B651D6-E1F2-41E7-B29B-9A942424F3DA}">
-  <dimension ref="A1:C20"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:C29"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="10.47265625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
     </row>
-    <row r="2" spans="1:3" s="5" customFormat="1" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:3" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>16</v>
       </c>
@@ -1149,7 +1236,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="8">
         <v>1</v>
       </c>
@@ -1160,7 +1247,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
         <v>2</v>
       </c>
@@ -1171,7 +1258,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="8">
         <v>3</v>
       </c>
@@ -1182,7 +1269,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="8">
         <v>4</v>
       </c>
@@ -1193,7 +1280,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="8">
         <v>5</v>
       </c>
@@ -1204,7 +1291,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
         <v>6</v>
       </c>
@@ -1215,7 +1302,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
         <v>7</v>
       </c>
@@ -1226,7 +1313,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
         <v>8</v>
       </c>
@@ -1237,7 +1324,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
         <v>9</v>
       </c>
@@ -1248,7 +1335,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="8">
         <v>10</v>
       </c>
@@ -1259,7 +1346,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="8">
         <v>11</v>
       </c>
@@ -1270,7 +1357,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="8">
         <v>12</v>
       </c>
@@ -1281,7 +1368,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="8">
         <v>13</v>
       </c>
@@ -1292,7 +1379,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="8">
         <v>14</v>
       </c>
@@ -1303,8 +1390,8 @@
         <v>42</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A17" s="11">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17" s="8">
         <v>15</v>
       </c>
       <c r="B17" s="6" t="s">
@@ -1314,8 +1401,8 @@
         <v>43</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A18" s="11">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A18" s="8">
         <v>16</v>
       </c>
       <c r="B18" s="6" t="s">
@@ -1325,8 +1412,8 @@
         <v>44</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A19" s="11">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A19" s="8">
         <v>17</v>
       </c>
       <c r="B19" s="6" t="s">
@@ -1336,8 +1423,45 @@
         <v>45</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A20" s="12"/>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C21" s="12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C23" s="11" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C24" s="11" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C25" s="11" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C26" s="11" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C27" s="11" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C28" s="11" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C29" s="11" t="s">
+        <v>152</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1349,17 +1473,17 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFD3CC65-B1DC-40CC-80A5-8E53941FB4A7}">
-  <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:C36"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="16.47265625" customWidth="1"/>
+    <col min="3" max="3" width="16.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
     </row>
-    <row r="2" spans="1:3" s="5" customFormat="1" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:3" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1367,7 +1491,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="8">
         <v>1</v>
       </c>
@@ -1378,7 +1502,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
         <v>2</v>
       </c>
@@ -1389,7 +1513,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="8">
         <v>3</v>
       </c>
@@ -1400,7 +1524,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="8">
         <v>4</v>
       </c>
@@ -1411,7 +1535,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="8">
         <v>5</v>
       </c>
@@ -1422,7 +1546,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
         <v>6</v>
       </c>
@@ -1433,7 +1557,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
         <v>7</v>
       </c>
@@ -1444,7 +1568,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
         <v>8</v>
       </c>
@@ -1455,7 +1579,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
         <v>9</v>
       </c>
@@ -1466,7 +1590,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="8">
         <v>10</v>
       </c>
@@ -1477,7 +1601,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="8">
         <v>11</v>
       </c>
@@ -1488,7 +1612,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="8">
         <v>12</v>
       </c>
@@ -1499,7 +1623,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="8">
         <v>13</v>
       </c>
@@ -1510,7 +1634,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="8">
         <v>14</v>
       </c>
@@ -1521,7 +1645,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="8">
         <v>15</v>
       </c>
@@ -1532,7 +1656,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="8">
         <v>16</v>
       </c>
@@ -1543,7 +1667,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
         <v>17</v>
       </c>
@@ -1554,7 +1678,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
         <v>18</v>
       </c>
@@ -1565,7 +1689,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="8">
         <v>19</v>
       </c>
@@ -1576,7 +1700,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="8">
         <v>20</v>
       </c>
@@ -1587,7 +1711,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="8">
         <v>21</v>
       </c>
@@ -1598,8 +1722,8 @@
         <v>66</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A24" s="11">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A24" s="8">
         <v>22</v>
       </c>
       <c r="B24" s="6" t="s">
@@ -1609,8 +1733,8 @@
         <v>67</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A25" s="11">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A25" s="8">
         <v>23</v>
       </c>
       <c r="B25" s="6" t="s">
@@ -1620,11 +1744,50 @@
         <v>68</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A26" s="12"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A27" s="12"/>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C27" s="12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C29" s="11" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C30" s="11" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C31" s="11" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C32" s="11" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C33" s="11" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C34" s="11" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="35" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C35" s="11" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="36" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C36" s="11" t="s">
+        <v>145</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1636,17 +1799,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46E14385-F8E9-4ECB-B0B5-CDB1847697B0}">
-  <dimension ref="A1:C29"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="15.1875" customWidth="1"/>
+    <col min="3" max="3" width="15.25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
     </row>
-    <row r="2" spans="1:3" s="5" customFormat="1" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:3" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
@@ -1654,7 +1817,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="3" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="8">
         <v>1</v>
       </c>
@@ -1665,7 +1828,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="4" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="8">
         <v>2</v>
       </c>
@@ -1676,7 +1839,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="5" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="8">
         <v>3</v>
       </c>
@@ -1687,7 +1850,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="6" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="8">
         <v>4</v>
       </c>
@@ -1698,7 +1861,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="7" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="8">
         <v>5</v>
       </c>
@@ -1709,7 +1872,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="8" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
         <v>6</v>
       </c>
@@ -1720,7 +1883,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="9" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
         <v>7</v>
       </c>
@@ -1731,7 +1894,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="10" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="8">
         <v>8</v>
       </c>
@@ -1742,7 +1905,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="11" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="8">
         <v>9</v>
       </c>
@@ -1753,7 +1916,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="12" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
         <v>10</v>
       </c>
@@ -1764,7 +1927,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="13" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="8">
         <v>11</v>
       </c>
@@ -1775,7 +1938,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="14" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
         <v>12</v>
       </c>
@@ -1786,7 +1949,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="15" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="8">
         <v>13</v>
       </c>
@@ -1797,7 +1960,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="16" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="8">
         <v>14</v>
       </c>
@@ -1808,7 +1971,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="17" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="8">
         <v>15</v>
       </c>
@@ -1819,7 +1982,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="18" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="8">
         <v>16</v>
       </c>
@@ -1830,7 +1993,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="19" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="8">
         <v>17</v>
       </c>
@@ -1841,7 +2004,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="20" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="8">
         <v>18</v>
       </c>
@@ -1852,7 +2015,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="21" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="8">
         <v>19</v>
       </c>
@@ -1863,7 +2026,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="22" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="8">
         <v>20</v>
       </c>
@@ -1874,8 +2037,8 @@
         <v>88</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="A23" s="11">
+    <row r="23" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A23" s="8">
         <v>21</v>
       </c>
       <c r="B23" s="2" t="s">
@@ -1885,8 +2048,8 @@
         <v>89</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="15.6" x14ac:dyDescent="0.6">
-      <c r="A24" s="11">
+    <row r="24" spans="1:3" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A24" s="8">
         <v>22</v>
       </c>
       <c r="B24" s="2" t="s">
@@ -1896,20 +2059,48 @@
         <v>90</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A25" s="12"/>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A26" s="12"/>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A27" s="12"/>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A28" s="12"/>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A29" s="12"/>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C26" s="12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C27" s="12"/>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C28" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C29" s="11" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C30" s="11" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C31" s="11" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C32" s="11" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="33" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C33" s="11" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="34" spans="3:3" x14ac:dyDescent="0.2">
+      <c r="C34" s="11" t="s">
+        <v>128</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1921,18 +2112,18 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F2A6B05-006C-44F8-95B1-390556A2FDA7}">
-  <dimension ref="A1:C34"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:C44"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="2" max="2" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" customWidth="1"/>
+    <col min="2" max="2" width="8.875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
     </row>
-    <row r="2" spans="1:3" s="5" customFormat="1" ht="15.6" x14ac:dyDescent="0.6">
+    <row r="2" spans="1:3" s="5" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="B2" s="4" t="s">
         <v>1</v>
       </c>
@@ -1940,7 +2131,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="8">
         <v>1</v>
       </c>
@@ -1951,7 +2142,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="8">
         <v>2</v>
       </c>
@@ -1962,7 +2153,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="8">
         <v>3</v>
       </c>
@@ -1973,7 +2164,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="8">
         <v>4</v>
       </c>
@@ -1984,7 +2175,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="8">
         <v>5</v>
       </c>
@@ -1995,7 +2186,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="8">
         <v>6</v>
       </c>
@@ -2006,7 +2197,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="8">
         <v>7</v>
       </c>
@@ -2017,7 +2208,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="8">
         <v>8</v>
       </c>
@@ -2028,7 +2219,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:3" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="8">
         <v>9</v>
       </c>
@@ -2039,7 +2230,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="8">
         <v>10</v>
       </c>
@@ -2050,7 +2241,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="8">
         <v>11</v>
       </c>
@@ -2061,7 +2252,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="8">
         <v>12</v>
       </c>
@@ -2072,7 +2263,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="8">
         <v>13</v>
       </c>
@@ -2083,7 +2274,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="8">
         <v>14</v>
       </c>
@@ -2094,7 +2285,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="8">
         <v>15</v>
       </c>
@@ -2105,7 +2296,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="8">
         <v>16</v>
       </c>
@@ -2116,7 +2307,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="8">
         <v>17</v>
       </c>
@@ -2127,7 +2318,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="8">
         <v>18</v>
       </c>
@@ -2138,7 +2329,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="8">
         <v>19</v>
       </c>
@@ -2149,7 +2340,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="8">
         <v>20</v>
       </c>
@@ -2160,7 +2351,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="8">
         <v>21</v>
       </c>
@@ -2171,7 +2362,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="8">
         <v>22</v>
       </c>
@@ -2182,7 +2373,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="8">
         <v>23</v>
       </c>
@@ -2193,7 +2384,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="8">
         <v>24</v>
       </c>
@@ -2204,7 +2395,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="8">
         <v>25</v>
       </c>
@@ -2215,7 +2406,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="8">
         <v>26</v>
       </c>
@@ -2226,7 +2417,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="8">
         <v>27</v>
       </c>
@@ -2237,7 +2428,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="8">
         <v>28</v>
       </c>
@@ -2248,7 +2439,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="8">
         <v>29</v>
       </c>
@@ -2259,8 +2450,8 @@
         <v>119</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A32" s="11">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A32" s="8">
         <v>30</v>
       </c>
       <c r="B32" s="1" t="s">
@@ -2270,8 +2461,8 @@
         <v>120</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A33" s="11">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="8">
         <v>31</v>
       </c>
       <c r="B33" s="1" t="s">
@@ -2281,8 +2472,50 @@
         <v>121</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.45">
-      <c r="A34" s="12"/>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C35" s="12" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C37" s="11" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C38" s="11" t="s">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C39" s="11" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C40" s="11" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C41" s="11" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C42" s="11" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C43" s="11" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="C44" s="11" t="s">
+        <v>137</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>